<commit_message>
revert(repository): 還原 sfw JOIN 回 GROUP BY（SQL 語法問題）
OUTER APPLY 在 Oracle 後接 LEFT JOIN 時產生 ORA-00933，
改在 Java 層處理去重，SQL 維持原樣。

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tiptop_MO.xlsx
+++ b/Tiptop_MO.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -16,6 +16,8 @@
     <sheet name="作業資料(ecd_file)" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="料件資料主檔(ima_file)_V2" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="部門名稱資料(gem_file)" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="工單完工入庫單頭檔(sfu_file)" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="工單完工入庫單身檔(sfv_file)" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -27,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3340" uniqueCount="1794">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3646" uniqueCount="1933">
   <si>
     <r>
       <rPr>
@@ -79,519 +81,81 @@
     <t xml:space="preserve">工單型態</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">工單型態
+    <t xml:space="preserve">工單型態
 儲存該工單所屬類別型態
-正確值 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">1/2/5/7/11/12/13/15
-1: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">一般工單
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">5: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">再加工工單
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">7: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">委外工單
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">8: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">重工委外工單 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">#Add By Snow
-11: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">拆件式工單
+正確值 1/2/5/7/11/12/13/15
+1: 一般工單
+5: 再加工工單
+7: 委外工單
+8: 重工委外工單 #Add By Snow
+11: 拆件式工單
 13: 預測工單
 15: 試產工單
 </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">工單型態 
+  </si>
+  <si>
+    <t xml:space="preserve">工單型態 
 儲存該工單所屬類別型態 
-正確值 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">1/2/5/7/11/12/13/15 
-1: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">一般工單  
+正確值 1/2/5/7/11/12/13/15 
+1: 一般工單  
+5: 再加工工單  
+7: 委外工單  
+8: 重工委外工單   #Add By Snow 
+11: 拆件式工單 
+13: 預測工單 
+15: 試產工單 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfb03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">varchar2(24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">在製品會計科目</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans TC"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">在製品會計科目  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">aag01</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">sfb04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">varchar2(1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">工單狀態</t>
+  </si>
+  <si>
+    <t xml:space="preserve">工單狀態
+儲存該工單目前處理階段狀況
+正確值 1/2/3/4/5/6/7/8
+1: 確認生產工單(firm plan)
+2: 工單已發放,料表尚未列印
+3: 工單已發放,料表已列印
+4: 工單已發料
+5: 在製過程中
+6: 工單已完工,進入F.Q.C
+7: 完工入庫
+8: 結案
 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">5: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">再加工工單  
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">7: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">委外工單  
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">8: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">重工委外工單   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">#Add By Snow 
-11: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">拆件式工單 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">13: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">預測工單 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">15: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">試產工單 </t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">sfb03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">varchar2(24)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">在製品會計科目</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">在製品會計科目  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">aag01</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">sfb04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">varchar2(1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">工單狀態</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">工單狀態
-儲存該工單目前處理階段狀況
-正確值 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">1/2/3/4/5/6/7/8
-1: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">確認生產工單</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">(firm plan)
-2: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">工單已發放</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">料表尚未列印
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">3: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">工單已發放</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">料表已列印
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">4: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">工單已發料
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">5: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">在製過程中
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">6: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">工單已完工</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">進入</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">F.Q.C
-7: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">完工入庫
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">8: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">結案
-</t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">工單狀態 
@@ -710,8 +274,26 @@
         <family val="2"/>
         <charset val="136"/>
       </rPr>
-      <t xml:space="preserve">儲存該工單將投入生產料件時所用的製程編
-號</t>
+      <t xml:space="preserve">儲存該工單將投入生產料件時所用的製程編</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans TC"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">號</t>
     </r>
   </si>
   <si>
@@ -2182,36 +1764,39 @@
     <t xml:space="preserve">備料檔產生否</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">備料檔產生否
+    <t xml:space="preserve">備料檔產生否
 儲存該工單是否已產生備料資料
-正確值 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">Y/N
-Y: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">該工單已產生備料資料
-</t>
+正確值 Y/N
+Y: 該工單已產生備料資料
+N: 該工單尚未產生備料資料</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans TC"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">備料檔產生否 儲存該工單是否已產生備料資料 正確值 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">Y/N Y: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans TC"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">該工單已產生備料資料 </t>
     </r>
     <r>
       <rPr>
@@ -2233,108 +1818,17 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">備料檔產生否 儲存該工單是否已產生備料資料 正確值 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">Y/N Y: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">該工單已產生備料資料 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">N: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">該工單尚未產生備料資料</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">sfb24</t>
   </si>
   <si>
     <t xml:space="preserve">製程追蹤檔產生否</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">製程追蹤檔產生否
+    <t xml:space="preserve">製程追蹤檔產生否
 儲存該工單是否已產生製程追蹤資料
-正確值 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">Y/N
-Y: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">該工單已產生製程追蹤資料
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">N: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">該工單尚未產生製程追蹤資料</t>
-    </r>
+正確值 Y/N
+Y: 該工單已產生製程追蹤資料
+N: 該工單尚未產生製程追蹤資料</t>
   </si>
   <si>
     <r>
@@ -3123,9 +2617,45 @@
         <family val="2"/>
         <charset val="136"/>
       </rPr>
-      <t xml:space="preserve">儲存該工單自上次料需求計劃後，如有變動
-時，則需在此備註
-提供 </t>
+      <t xml:space="preserve">儲存該工單自上次料需求計劃後，如有變動</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans TC"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">時，則需在此備註</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans TC"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">提供 </t>
     </r>
     <r>
       <rPr>
@@ -3253,104 +2783,15 @@
     <t xml:space="preserve">完工方式</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">完工方式
+    <t xml:space="preserve">完工方式
 儲存該工單在料帳上，使用撿料及發料系統
 或使用領料及事後扣帳系統
-正確值 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">1/2
-1: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">撿料及發料系統
+正確值 1/2
+1: 撿料及發料系統
+Picking List 與 Push System
+2: 領料及事後扣帳系統
+Pull List 與 Backflush System
 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">Picking List </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">與 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">Push System
-2: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">領料及事後扣帳系統
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">Pull List </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">與 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">Backflush System
-</t>
-    </r>
   </si>
   <si>
     <r>
@@ -3874,63 +3315,9 @@
         <charset val="136"/>
       </rPr>
       <t xml:space="preserve">委外工單對委外採購單型態為一對一
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">2.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">委外工單對委外採購單型態為一對多
-預設 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">'1'
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">兩者的差別在於</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans TC"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t xml:space="preserve">資料的一致性
+2.委外工單對委外採購單型態為一對多
+預設 '1'
+兩者的差別在於,資料的一致性
 </t>
     </r>
   </si>
@@ -34312,6 +33699,423 @@
   </si>
   <si>
     <t xml:space="preserve">gemoriu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">工單完工入庫單頭檔(sfu_file)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">類別</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.入庫  2.入庫退回 3.重複性生產入庫</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">入庫日期</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">varchar2(16)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">部門</t>
+  </si>
+  <si>
+    <t xml:space="preserve">部門     gem01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">理由</t>
+  </si>
+  <si>
+    <t xml:space="preserve">理由     azf01,azf02='2'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">專案編號</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PBI#     sfc01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">耗材單號</t>
+  </si>
+  <si>
+    <t xml:space="preserve">耗材單號 sfp01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfupost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">過帳否</t>
+  </si>
+  <si>
+    <t xml:space="preserve">過帳否(Y/N/X)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuuser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfugrup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfumodu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfudate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuconf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuud15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuplant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfulegal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuoriu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfuorig</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfumksg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfu17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WIP單號</t>
+  </si>
+  <si>
+    <t xml:space="preserve">工單完工入庫單身檔(sfv_file)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">入庫編號</t>
+  </si>
+  <si>
+    <t xml:space="preserve">入庫編號 sfu01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">料號</t>
+  </si>
+  <si>
+    <t xml:space="preserve">料號     ima01(sfa03)(img01)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">倉庫</t>
+  </si>
+  <si>
+    <t xml:space="preserve">倉庫     imd01(img02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">儲位</t>
+  </si>
+  <si>
+    <t xml:space="preserve">儲位     ime01(img03)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">批號</t>
+  </si>
+  <si>
+    <t xml:space="preserve">批號           img04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">庫存單位       ima25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">入庫量</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">工單單號</t>
+  </si>
+  <si>
+    <t xml:space="preserve">工單編號       sfb01(ASR此欄是計劃料號)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">備註 (委外工單入庫時輸入發票號碼)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">當月是否入聯產品否</t>
+  </si>
+  <si>
+    <t xml:space="preserve">當月是否入聯產品否 #6872系統維護</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASR-報工單號 (asrt320)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asft620 - 報工單號</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">單位一</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">單位一換算率(與生產單位)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">單位一數量</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">單位二</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">單位二換算率(與生產單位)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">單位二數量</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv930</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">專案代號</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WBS編碼</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvud15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvplant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfvlegal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QC判定結果編碼</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sfv47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QC判定結果項次</t>
   </si>
 </sst>
 </file>
@@ -34590,37 +34394,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -34756,7 +34560,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="122" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="62" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
@@ -34808,7 +34612,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="146" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="98" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
         <v>17</v>
       </c>
@@ -34860,7 +34664,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="38" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="26" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
         <v>27</v>
       </c>
@@ -34886,7 +34690,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="26" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
         <v>32</v>
       </c>
@@ -34912,7 +34716,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="26" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="38" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
         <v>36</v>
       </c>
@@ -34984,7 +34788,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="26" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
         <v>48</v>
       </c>
@@ -35036,7 +34840,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="26" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
         <v>56</v>
       </c>
@@ -35466,7 +35270,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="62" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="38" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
         <v>118</v>
       </c>
@@ -35492,7 +35296,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="62" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="38" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
         <v>122</v>
       </c>
@@ -35584,7 +35388,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="26" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
         <v>134</v>
       </c>
@@ -35766,7 +35570,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="62" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="74" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
         <v>164</v>
       </c>
@@ -35818,7 +35622,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="50" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="38" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
         <v>173</v>
       </c>
@@ -35844,7 +35648,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="62" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="74" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
         <v>177</v>
       </c>
@@ -35870,7 +35674,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="74" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="86" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
         <v>181</v>
       </c>
@@ -35922,7 +35726,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="110" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="96" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
         <v>189</v>
       </c>
@@ -36350,7 +36154,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="74" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="50" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
         <v>242</v>
       </c>
@@ -36454,7 +36258,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="26" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
         <v>257</v>
       </c>
@@ -37560,6 +37364,616 @@
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,標準"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,標準"&amp;12頁 &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A2:D54"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="17" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="2" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>1854</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>1855</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>1856</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>1857</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>1858</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>1859</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>1860</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>1861</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>1862</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>1863</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>1864</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>1865</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>1866</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>1867</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>1868</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>1869</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>1870</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>1871</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>278</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>1170</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>1872</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
+        <v>1873</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>1874</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>1875</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>1876</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>1877</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
+        <v>1878</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>233</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>1879</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
+        <v>1880</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="0" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
+        <v>1881</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>1882</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
+        <v>1883</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>1884</v>
+      </c>
+      <c r="D19" s="0" t="s">
+        <v>1885</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>1886</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>805</v>
+      </c>
+      <c r="D20" s="0" t="s">
+        <v>1887</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
+        <v>1888</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
+        <v>1889</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="0" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="s">
+        <v>1890</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>769</v>
+      </c>
+      <c r="C23" s="0" t="s">
+        <v>770</v>
+      </c>
+      <c r="D23" s="0" t="s">
+        <v>1891</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="s">
+        <v>1892</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>278</v>
+      </c>
+      <c r="C24" s="0" t="s">
+        <v>1893</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
+        <v>1894</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>431</v>
+      </c>
+      <c r="C25" s="0" t="s">
+        <v>1895</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="s">
+        <v>1896</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="0" t="s">
+        <v>1897</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="s">
+        <v>1898</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>278</v>
+      </c>
+      <c r="C27" s="0" t="s">
+        <v>1899</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>1900</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>431</v>
+      </c>
+      <c r="C28" s="0" t="s">
+        <v>1901</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
+        <v>1902</v>
+      </c>
+      <c r="B29" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C29" s="0" t="s">
+        <v>1903</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>1904</v>
+      </c>
+      <c r="B30" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" s="0" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="s">
+        <v>1905</v>
+      </c>
+      <c r="B31" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C31" s="0" t="s">
+        <v>1906</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="s">
+        <v>1907</v>
+      </c>
+      <c r="B32" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>1908</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0" t="s">
+        <v>1909</v>
+      </c>
+      <c r="B33" s="0" t="s">
+        <v>278</v>
+      </c>
+      <c r="C33" s="0" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="s">
+        <v>1910</v>
+      </c>
+      <c r="B34" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C34" s="0" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="s">
+        <v>1911</v>
+      </c>
+      <c r="B35" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="C35" s="0" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="s">
+        <v>1912</v>
+      </c>
+      <c r="B36" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C36" s="0" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="0" t="s">
+        <v>1913</v>
+      </c>
+      <c r="B37" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C37" s="0" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="0" t="s">
+        <v>1914</v>
+      </c>
+      <c r="B38" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C38" s="0" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="0" t="s">
+        <v>1915</v>
+      </c>
+      <c r="B39" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C39" s="0" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="0" t="s">
+        <v>1916</v>
+      </c>
+      <c r="B40" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C40" s="0" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="s">
+        <v>1917</v>
+      </c>
+      <c r="B41" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C41" s="0" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="s">
+        <v>1918</v>
+      </c>
+      <c r="B42" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C42" s="0" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="0" t="s">
+        <v>1919</v>
+      </c>
+      <c r="B43" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C43" s="0" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0" t="s">
+        <v>1920</v>
+      </c>
+      <c r="B44" s="0" t="s">
+        <v>298</v>
+      </c>
+      <c r="C44" s="0" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="0" t="s">
+        <v>1921</v>
+      </c>
+      <c r="B45" s="0" t="s">
+        <v>298</v>
+      </c>
+      <c r="C45" s="0" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="0" t="s">
+        <v>1922</v>
+      </c>
+      <c r="B46" s="0" t="s">
+        <v>298</v>
+      </c>
+      <c r="C46" s="0" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="0" t="s">
+        <v>1923</v>
+      </c>
+      <c r="B47" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C47" s="0" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="0" t="s">
+        <v>1924</v>
+      </c>
+      <c r="B48" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C48" s="0" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="0" t="s">
+        <v>1925</v>
+      </c>
+      <c r="B49" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C49" s="0" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="0" t="s">
+        <v>1926</v>
+      </c>
+      <c r="B50" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C50" s="0" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="0" t="s">
+        <v>1927</v>
+      </c>
+      <c r="B51" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C51" s="0" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="0" t="s">
+        <v>1928</v>
+      </c>
+      <c r="B52" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C52" s="0" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="0" t="s">
+        <v>1929</v>
+      </c>
+      <c r="B53" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C53" s="0" t="s">
+        <v>1930</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="0" t="s">
+        <v>1931</v>
+      </c>
+      <c r="B54" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" s="0" t="s">
+        <v>1932</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,標準"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,標準"&amp;12頁 &amp;P</oddFooter>
@@ -46454,4 +46868,544 @@
     <oddFooter>&amp;C&amp;"Times New Roman,標準"&amp;12頁 &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A2:D49"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="17" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="2" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>1794</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>1795</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>1796</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>1797</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>1798</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>1799</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>1801</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>1802</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>1803</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>1804</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>1805</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>1806</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>1807</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>1808</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>1809</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>1810</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
+        <v>1811</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>1812</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>212</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>1813</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
+        <v>1814</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>1815</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>1816</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
+        <v>1817</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="0" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
+        <v>1818</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>1819</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
+        <v>1820</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>1821</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>1822</v>
+      </c>
+      <c r="D20" s="0" t="s">
+        <v>1823</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="s">
+        <v>1824</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="s">
+        <v>1825</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" s="0" t="s">
+        <v>1782</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="s">
+        <v>1826</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" s="0" t="s">
+        <v>1784</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="s">
+        <v>1827</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" s="0" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
+        <v>1828</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="0" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="s">
+        <v>1829</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>232</v>
+      </c>
+      <c r="C26" s="0" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="s">
+        <v>1830</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C27" s="0" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>1831</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28" s="0" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
+        <v>1832</v>
+      </c>
+      <c r="B29" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C29" s="0" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>1833</v>
+      </c>
+      <c r="B30" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C30" s="0" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="s">
+        <v>1834</v>
+      </c>
+      <c r="B31" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C31" s="0" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="s">
+        <v>1835</v>
+      </c>
+      <c r="B32" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="0" t="s">
+        <v>1836</v>
+      </c>
+      <c r="B33" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C33" s="0" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="s">
+        <v>1837</v>
+      </c>
+      <c r="B34" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="C34" s="0" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B35" s="0" t="s">
+        <v>298</v>
+      </c>
+      <c r="C35" s="0" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="s">
+        <v>1839</v>
+      </c>
+      <c r="B36" s="0" t="s">
+        <v>298</v>
+      </c>
+      <c r="C36" s="0" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="0" t="s">
+        <v>1840</v>
+      </c>
+      <c r="B37" s="0" t="s">
+        <v>298</v>
+      </c>
+      <c r="C37" s="0" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="0" t="s">
+        <v>1841</v>
+      </c>
+      <c r="B38" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C38" s="0" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="0" t="s">
+        <v>1842</v>
+      </c>
+      <c r="B39" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C39" s="0" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="0" t="s">
+        <v>1843</v>
+      </c>
+      <c r="B40" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C40" s="0" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="s">
+        <v>1844</v>
+      </c>
+      <c r="B41" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C41" s="0" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="0" t="s">
+        <v>1845</v>
+      </c>
+      <c r="B42" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C42" s="0" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="0" t="s">
+        <v>1846</v>
+      </c>
+      <c r="B43" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C43" s="0" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0" t="s">
+        <v>1847</v>
+      </c>
+      <c r="B44" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C44" s="0" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="0" t="s">
+        <v>1848</v>
+      </c>
+      <c r="B45" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C45" s="0" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="0" t="s">
+        <v>1849</v>
+      </c>
+      <c r="B46" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C46" s="0" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="0" t="s">
+        <v>1850</v>
+      </c>
+      <c r="B47" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C47" s="0" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="0" t="s">
+        <v>1851</v>
+      </c>
+      <c r="B48" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C48" s="0" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="0" t="s">
+        <v>1852</v>
+      </c>
+      <c r="B49" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C49" s="0" t="s">
+        <v>1853</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,標準"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,標準"&amp;12頁 &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>